<commit_message>
Safety: handle real-export quirks, E/R/Unclassified classes, compact load bar
- Ignore blank/formula-only rows; '-', '$ -', '(blank)', N/A read as zero/blank;
  parentheses negatives; report only real unreadable cells with up to 5 examples
- Accident Class A-D, E (Ground), R (NG), Unclassified (blank); unknown values shown raw
- Optional columns Assigned To, Comments (tracker + drawer), SUB DATE REPORTED, Documentation
- Load panel collapses to a one-line status bar (state remembered); Presentation mode
- Demo data gains E/R/unclassified records and optional columns; Power BI kit updated
</commit_message>
<xml_diff>
--- a/dashboards/safety/asmis_template.xlsx
+++ b/dashboards/safety/asmis_template.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS1"/>
+  <dimension ref="A1:AW1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -644,6 +644,26 @@
       <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Summary</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>SUB DATE REPORTED</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>Documentation</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>Comments</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>Assigned To</t>
         </is>
       </c>
     </row>

</xml_diff>